<commit_message>
fix: :bug: fix eval checkpoint script
</commit_message>
<xml_diff>
--- a/GRPO/Evaluation/metrics_summary.xlsx
+++ b/GRPO/Evaluation/metrics_summary.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,19 +25,26 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font/>
     <font>
-      <b val="1"/>
+      <color rgb="00008000"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0090EE90"/>
+        <bgColor rgb="0090EE90"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +52,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,108 +426,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>checkpoint</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>aime_acc</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>aimo_acc</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>art_acc</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>art_f1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>art_precision</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>art_recall</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>copa_guess_effect_acc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>copa_guess_effect_f1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>copa_guess_effect_precision</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>copa_guess_effect_recall</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>goemotion_acc</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>goemotion_f1</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>goemotion_hamming_acc</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>goemotion_precision</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>goemotion_recall</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>gsm8k_acc</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>better_metrics_than_raw</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>better_datasets_than_raw</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>qwen2.5-14B (Raw)</t>
         </is>
@@ -538,109 +489,59 @@
         <v>0.4819</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8114</v>
-      </c>
-      <c r="E2" t="n">
         <v>0.8113</v>
       </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>0.8124</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.8119</v>
+        <v>0.3365</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.903</v>
       </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="n">
-        <v>0.2591</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.3756</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.2604</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.3436</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.4141</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.903</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>checkpoint-512</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>0.1667</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>0.494</v>
       </c>
       <c r="D3" t="n">
         <v>0.8028999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8028999999999999</v>
+        <v>0.9196</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8036</v>
+        <v>0.3193</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8033</v>
+        <v>0.8969</v>
       </c>
       <c r="H3" t="n">
-        <v>0.914</v>
+        <v>0.198</v>
       </c>
       <c r="I3" t="n">
-        <v>0.9196</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8978</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.9425</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.2215</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.3582</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.2224</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.3176</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.4106</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.8969</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>checkpoint-1024</t>
         </is>
@@ -648,60 +549,33 @@
       <c r="B4" t="n">
         <v>0.0667</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>0.506</v>
       </c>
       <c r="D4" t="n">
         <v>0.8048</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8048</v>
+        <v>0.9129</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8052</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.8052</v>
+        <v>0.3239</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.903</v>
       </c>
       <c r="H4" t="n">
-        <v>0.908</v>
+        <v>0.2027</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9129</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>0.9026</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.9234</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.2335</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.3653</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.2346</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.3264</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.4146</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.903</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>checkpoint-1536</t>
         </is>
@@ -712,57 +586,30 @@
       <c r="C5" t="n">
         <v>0.4458</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>0.8179</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8179</v>
+        <v>0.9118000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8186</v>
+        <v>0.3279</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8183</v>
+        <v>0.9022</v>
       </c>
       <c r="H5" t="n">
-        <v>0.906</v>
+        <v>0.2058</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9118000000000001</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8934</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.2257</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.3618</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.2279</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.3216</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.4135</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.9022</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>checkpoint-2048</t>
         </is>
@@ -770,60 +617,33 @@
       <c r="B6" t="n">
         <v>0.1333</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>0.494</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8107</v>
+        <v>0.8106</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8106</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.8126</v>
+        <v>0.9193</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0.3366</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8115</v>
+        <v>0.8954</v>
       </c>
       <c r="H6" t="n">
-        <v>0.914</v>
+        <v>0.2066</v>
       </c>
       <c r="I6" t="n">
-        <v>0.9193</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9006999999999999</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.9387</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.2497</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.2524</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.3388</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.4198</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.8954</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>checkpoint-2560</t>
         </is>
@@ -831,60 +651,33 @@
       <c r="B7" t="n">
         <v>0.1</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2" t="n">
         <v>0.5181</v>
       </c>
-      <c r="D7" t="n">
-        <v>0.8139999999999999</v>
+      <c r="D7" s="2" t="n">
+        <v>0.8139</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8139</v>
+        <v>0.9179</v>
       </c>
       <c r="F7" t="n">
-        <v>0.8161</v>
+        <v>0.332</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8148</v>
+        <v>0.8961</v>
       </c>
       <c r="H7" t="n">
-        <v>0.912</v>
+        <v>0.2027</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9179</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
-        <v>0.8945</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.9425</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.2342</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.3719</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.2371</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.3326</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.4219</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.8961</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>checkpoint-3072</t>
         </is>
@@ -892,86 +685,128 @@
       <c r="B8" t="n">
         <v>0.1</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="2" t="n">
         <v>0.5301</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8087</v>
+        <v>0.8086</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8086</v>
+        <v>0.9179</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8114</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.8096</v>
+        <v>0.3282</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.906</v>
       </c>
       <c r="H8" t="n">
-        <v>0.912</v>
+        <v>0.2011</v>
       </c>
       <c r="I8" t="n">
-        <v>0.9179</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8945</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.9425</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.2377</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.371</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.2408</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.332</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.4203</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.906</v>
-      </c>
-      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>checkpoint-3584</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.0667</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.5301</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.8073</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9094</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.3249</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.2121</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>checkpoint-4096</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.8124</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9257</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.3285</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.9067</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.2207</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>checkpoint-4608(best)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.4819</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.8077</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9257</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>0.8946</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.2066</v>
+      </c>
+      <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>checkpoint-3584</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="n">
-        <v>0.903</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" t="n">
+      <c r="J11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>